<commit_message>
Daily EthioJobs tracker update 2026-09-24
</commit_message>
<xml_diff>
--- a/ethiojobs_tracker.xlsx
+++ b/ethiojobs_tracker.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U301"/>
+  <dimension ref="A1:U303"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -29055,6 +29055,205 @@
         </is>
       </c>
     </row>
+    <row r="302">
+      <c r="A302" t="inlineStr">
+        <is>
+          <t>QfJKSBO3jf</t>
+        </is>
+      </c>
+      <c r="B302" t="inlineStr">
+        <is>
+          <t>Senior Sales Officer</t>
+        </is>
+      </c>
+      <c r="C302" t="inlineStr">
+        <is>
+          <t>COMMERCIAL NOMINEES PLC</t>
+        </is>
+      </c>
+      <c r="D302" t="inlineStr">
+        <is>
+          <t>Sales and Marketing</t>
+        </is>
+      </c>
+      <c r="E302" t="inlineStr">
+        <is>
+          <t>Addis Ababa</t>
+        </is>
+      </c>
+      <c r="F302" t="inlineStr">
+        <is>
+          <t>Office</t>
+        </is>
+      </c>
+      <c r="G302" t="inlineStr">
+        <is>
+          <t>Junior Level(1-3 years)</t>
+        </is>
+      </c>
+      <c r="H302" t="inlineStr">
+        <is>
+          <t>Full time</t>
+        </is>
+      </c>
+      <c r="I302" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J302" t="inlineStr">
+        <is>
+          <t>, work experience, or other evidence ) submitted during employment/registration will result in legal accountability</t>
+        </is>
+      </c>
+      <c r="K302" t="inlineStr">
+        <is>
+          <t>3-5 years</t>
+        </is>
+      </c>
+      <c r="L302" t="inlineStr">
+        <is>
+          <t>Sales; Excellent communication and interpersonal skills.; Desired Skill; sals; Excellent communication and interpersonal skills.</t>
+        </is>
+      </c>
+      <c r="O302" t="inlineStr">
+        <is>
+          <t>October 1st, 2026</t>
+        </is>
+      </c>
+      <c r="P302" t="inlineStr">
+        <is>
+          <t>Applicants who meet the minimum requirements mentioned above can register through Ethiojobs or by sending your application to: cnplcvacancy@gmail.com by Specifying Job position and vacancy number clearly in the subject line of your email. Please also attached the following documents: Updated CV and all supporting documents, Work experience from non Government organizations must be supported by proof of employment tax payment, grade 8 completion certificate and "To whom it may concern letter" from your current employer
+Forgery liability: any falsified documents ( Education, work experience, or other evidence ) submitted during employment/registration will result in legal accountability
+Perks + Benefits
+Fuel
+Housing
+Medical Allowance</t>
+        </is>
+      </c>
+      <c r="Q302" t="inlineStr">
+        <is>
+          <t>https://ethiojobs.net/job/QfJKSBO3jf-senior-sales-officer</t>
+        </is>
+      </c>
+      <c r="R302" t="inlineStr">
+        <is>
+          <t>EthioJobs</t>
+        </is>
+      </c>
+      <c r="S302" t="inlineStr">
+        <is>
+          <t>15 minutes ago by</t>
+        </is>
+      </c>
+      <c r="T302" t="inlineStr">
+        <is>
+          <t>2026-09-24 10:45:35 UTC</t>
+        </is>
+      </c>
+      <c r="U302" t="inlineStr">
+        <is>
+          <t>dom_render</t>
+        </is>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="inlineStr">
+        <is>
+          <t>ozf3ombEhD</t>
+        </is>
+      </c>
+      <c r="B303" t="inlineStr">
+        <is>
+          <t>Social Workers – Child Protection (CP) &amp; Gender-Based Violence (GBV)</t>
+        </is>
+      </c>
+      <c r="C303" t="inlineStr">
+        <is>
+          <t>HELP GENERATION</t>
+        </is>
+      </c>
+      <c r="D303" t="inlineStr">
+        <is>
+          <t>Social Sciences and Com...</t>
+        </is>
+      </c>
+      <c r="E303" t="inlineStr">
+        <is>
+          <t>Afar</t>
+        </is>
+      </c>
+      <c r="F303" t="inlineStr">
+        <is>
+          <t>Office</t>
+        </is>
+      </c>
+      <c r="G303" t="inlineStr">
+        <is>
+          <t>Junior Level(1-3 years)</t>
+        </is>
+      </c>
+      <c r="H303" t="inlineStr">
+        <is>
+          <t>Contract</t>
+        </is>
+      </c>
+      <c r="I303" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="J303" t="inlineStr">
+        <is>
+          <t>Bachelor's degree</t>
+        </is>
+      </c>
+      <c r="K303" t="inlineStr">
+        <is>
+          <t>1-3 years</t>
+        </is>
+      </c>
+      <c r="L303" t="inlineStr">
+        <is>
+          <t>Psychology, Social Work, Gender Studies, Law</t>
+        </is>
+      </c>
+      <c r="O303" t="inlineStr">
+        <is>
+          <t>September 30th, 2026</t>
+        </is>
+      </c>
+      <c r="P303" t="inlineStr">
+        <is>
+          <t>Interested and qualified applicants who meet the above requirements are invited to submit their updated CV and a cover letter through Ethiojobs by clicking the "Apply" button within the specified timeframe. Please ensure your application clearly indicates your preferred woreda (Berhale, Dallol, or Koneba).</t>
+        </is>
+      </c>
+      <c r="Q303" t="inlineStr">
+        <is>
+          <t>https://ethiojobs.net/job/ozf3ombEhD-social-workers-child-protection-cp-gender-based-violence-gbv</t>
+        </is>
+      </c>
+      <c r="R303" t="inlineStr">
+        <is>
+          <t>EthioJobs</t>
+        </is>
+      </c>
+      <c r="S303" t="inlineStr">
+        <is>
+          <t>31 minutes ago by</t>
+        </is>
+      </c>
+      <c r="T303" t="inlineStr">
+        <is>
+          <t>2026-09-24 10:45:39 UTC</t>
+        </is>
+      </c>
+      <c r="U303" t="inlineStr">
+        <is>
+          <t>dom_render</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:U1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -29067,7 +29266,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -29098,6 +29297,19 @@
       </c>
       <c r="C2" t="n">
         <v>300</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-09-24 10:45:40 UTC</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" t="n">
+        <v>302</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily EthioJobs tracker update 2026-09-27
</commit_message>
<xml_diff>
--- a/ethiojobs_tracker.xlsx
+++ b/ethiojobs_tracker.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U476"/>
+  <dimension ref="A1:U483"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -45665,6 +45665,625 @@
         </is>
       </c>
     </row>
+    <row r="477">
+      <c r="A477" t="inlineStr">
+        <is>
+          <t>oaGimTgmqK</t>
+        </is>
+      </c>
+      <c r="B477" t="inlineStr">
+        <is>
+          <t>Project Health, Safety and Environment(HSE) Officer</t>
+        </is>
+      </c>
+      <c r="C477" t="inlineStr">
+        <is>
+          <t>TEMER PROPERTIES</t>
+        </is>
+      </c>
+      <c r="D477" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="E477" t="inlineStr">
+        <is>
+          <t>Addis Ababa</t>
+        </is>
+      </c>
+      <c r="F477" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="G477" t="inlineStr">
+        <is>
+          <t>Junior Level(1-3 years)</t>
+        </is>
+      </c>
+      <c r="H477" t="inlineStr">
+        <is>
+          <t>Full time</t>
+        </is>
+      </c>
+      <c r="I477" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="K477" t="inlineStr">
+        <is>
+          <t>1-3 years</t>
+        </is>
+      </c>
+      <c r="L477" t="inlineStr">
+        <is>
+          <t>Attention to detail; Communication &amp; Negotiation; Teamwork and collaboration</t>
+        </is>
+      </c>
+      <c r="O477" t="inlineStr">
+        <is>
+          <t>October 7th, 2026</t>
+        </is>
+      </c>
+      <c r="P477" t="inlineStr">
+        <is>
+          <t>Interested candidates are invited to submit their CV: jobs@temerproperties.com. Please write “Project Health, Safety and Environment (HSE) Officer " in the subject line.</t>
+        </is>
+      </c>
+      <c r="Q477" t="inlineStr">
+        <is>
+          <t>https://ethiojobs.net/job/oaGimTgmqK-project-health-safety-and-environmenthse-officer</t>
+        </is>
+      </c>
+      <c r="R477" t="inlineStr">
+        <is>
+          <t>EthioJobs</t>
+        </is>
+      </c>
+      <c r="S477" t="inlineStr">
+        <is>
+          <t>19 hours ago by</t>
+        </is>
+      </c>
+      <c r="T477" t="inlineStr">
+        <is>
+          <t>2026-09-27 11:02:36 UTC</t>
+        </is>
+      </c>
+      <c r="U477" t="inlineStr">
+        <is>
+          <t>dom_render</t>
+        </is>
+      </c>
+    </row>
+    <row r="478">
+      <c r="A478" t="inlineStr">
+        <is>
+          <t>wd8Mrtu0Om</t>
+        </is>
+      </c>
+      <c r="B478" t="inlineStr">
+        <is>
+          <t>Junior Battery Swapper</t>
+        </is>
+      </c>
+      <c r="C478" t="inlineStr">
+        <is>
+          <t>DODAI MANUFACTURING PLC.</t>
+        </is>
+      </c>
+      <c r="D478" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="E478" t="inlineStr">
+        <is>
+          <t>Addis Ababa</t>
+        </is>
+      </c>
+      <c r="F478" t="inlineStr">
+        <is>
+          <t>Office</t>
+        </is>
+      </c>
+      <c r="G478" t="inlineStr">
+        <is>
+          <t>Junior Level(1-3 years)</t>
+        </is>
+      </c>
+      <c r="H478" t="inlineStr">
+        <is>
+          <t>Full time</t>
+        </is>
+      </c>
+      <c r="I478" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="L478" t="inlineStr">
+        <is>
+          <t>Customer Servce orienation; Excellent communication and interpersonal skills.; Organization &amp; Time Management</t>
+        </is>
+      </c>
+      <c r="O478" t="inlineStr">
+        <is>
+          <t>October 10th, 2026</t>
+        </is>
+      </c>
+      <c r="P478" t="inlineStr">
+        <is>
+          <t>To Apply Use this Link</t>
+        </is>
+      </c>
+      <c r="Q478" t="inlineStr">
+        <is>
+          <t>https://ethiojobs.net/job/wd8Mrtu0Om-junior-battery-swapper</t>
+        </is>
+      </c>
+      <c r="R478" t="inlineStr">
+        <is>
+          <t>EthioJobs</t>
+        </is>
+      </c>
+      <c r="S478" t="inlineStr">
+        <is>
+          <t>a day ago by</t>
+        </is>
+      </c>
+      <c r="T478" t="inlineStr">
+        <is>
+          <t>2026-09-27 11:02:39 UTC</t>
+        </is>
+      </c>
+      <c r="U478" t="inlineStr">
+        <is>
+          <t>dom_render</t>
+        </is>
+      </c>
+    </row>
+    <row r="479">
+      <c r="A479" t="inlineStr">
+        <is>
+          <t>FRXDnJ8yKj</t>
+        </is>
+      </c>
+      <c r="B479" t="inlineStr">
+        <is>
+          <t>Accountant</t>
+        </is>
+      </c>
+      <c r="C479" t="inlineStr">
+        <is>
+          <t>DODAI MANUFACTURING PLC.</t>
+        </is>
+      </c>
+      <c r="D479" t="inlineStr">
+        <is>
+          <t>Accounting and Finance</t>
+        </is>
+      </c>
+      <c r="E479" t="inlineStr">
+        <is>
+          <t>Addis Ababa</t>
+        </is>
+      </c>
+      <c r="F479" t="inlineStr">
+        <is>
+          <t>Office</t>
+        </is>
+      </c>
+      <c r="G479" t="inlineStr">
+        <is>
+          <t>Mid Level(3-5 years)</t>
+        </is>
+      </c>
+      <c r="H479" t="inlineStr">
+        <is>
+          <t>Full time</t>
+        </is>
+      </c>
+      <c r="I479" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="L479" t="inlineStr">
+        <is>
+          <t>Able to Properly Use Peachtree (Record, Post, close …Accounts); Knowledge of accounting principles; Strong skill in basic accounting and book keeping.; Accounts Payable &amp; Receivable</t>
+        </is>
+      </c>
+      <c r="O479" t="inlineStr">
+        <is>
+          <t>October 10th, 2026</t>
+        </is>
+      </c>
+      <c r="P479" t="inlineStr">
+        <is>
+          <t>To Apply this Link</t>
+        </is>
+      </c>
+      <c r="Q479" t="inlineStr">
+        <is>
+          <t>https://ethiojobs.net/job/FRXDnJ8yKj-accountant</t>
+        </is>
+      </c>
+      <c r="R479" t="inlineStr">
+        <is>
+          <t>EthioJobs</t>
+        </is>
+      </c>
+      <c r="S479" t="inlineStr">
+        <is>
+          <t>a day ago by</t>
+        </is>
+      </c>
+      <c r="T479" t="inlineStr">
+        <is>
+          <t>2026-09-27 11:02:43 UTC</t>
+        </is>
+      </c>
+      <c r="U479" t="inlineStr">
+        <is>
+          <t>dom_render</t>
+        </is>
+      </c>
+    </row>
+    <row r="480">
+      <c r="A480" t="inlineStr">
+        <is>
+          <t>iEQfaUfbgN</t>
+        </is>
+      </c>
+      <c r="B480" t="inlineStr">
+        <is>
+          <t>Junior Accountant</t>
+        </is>
+      </c>
+      <c r="C480" t="inlineStr">
+        <is>
+          <t>DODAI MANUFACTURING PLC.</t>
+        </is>
+      </c>
+      <c r="D480" t="inlineStr">
+        <is>
+          <t>Accounting and Finance</t>
+        </is>
+      </c>
+      <c r="E480" t="inlineStr">
+        <is>
+          <t>Addis Ababa</t>
+        </is>
+      </c>
+      <c r="F480" t="inlineStr">
+        <is>
+          <t>Office</t>
+        </is>
+      </c>
+      <c r="G480" t="inlineStr">
+        <is>
+          <t>Junior Level(1-3 years)</t>
+        </is>
+      </c>
+      <c r="H480" t="inlineStr">
+        <is>
+          <t>Full time</t>
+        </is>
+      </c>
+      <c r="I480" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="L480" t="inlineStr">
+        <is>
+          <t>Communication; Accounting; computer skill; accuracy</t>
+        </is>
+      </c>
+      <c r="O480" t="inlineStr">
+        <is>
+          <t>October 10th, 2026</t>
+        </is>
+      </c>
+      <c r="P480" t="inlineStr">
+        <is>
+          <t>To Apply Use this Link</t>
+        </is>
+      </c>
+      <c r="Q480" t="inlineStr">
+        <is>
+          <t>https://ethiojobs.net/job/iEQfaUfbgN-junior-accountant</t>
+        </is>
+      </c>
+      <c r="R480" t="inlineStr">
+        <is>
+          <t>EthioJobs</t>
+        </is>
+      </c>
+      <c r="S480" t="inlineStr">
+        <is>
+          <t>a day ago by</t>
+        </is>
+      </c>
+      <c r="T480" t="inlineStr">
+        <is>
+          <t>2026-09-27 11:02:46 UTC</t>
+        </is>
+      </c>
+      <c r="U480" t="inlineStr">
+        <is>
+          <t>dom_render</t>
+        </is>
+      </c>
+    </row>
+    <row r="481">
+      <c r="A481" t="inlineStr">
+        <is>
+          <t>WAhlweiNIf</t>
+        </is>
+      </c>
+      <c r="B481" t="inlineStr">
+        <is>
+          <t>Junior Customer Experience Officer</t>
+        </is>
+      </c>
+      <c r="C481" t="inlineStr">
+        <is>
+          <t>DODAI MANUFACTURING PLC.</t>
+        </is>
+      </c>
+      <c r="D481" t="inlineStr">
+        <is>
+          <t>Customer Service</t>
+        </is>
+      </c>
+      <c r="E481" t="inlineStr">
+        <is>
+          <t>Addis Ababa</t>
+        </is>
+      </c>
+      <c r="F481" t="inlineStr">
+        <is>
+          <t>Office</t>
+        </is>
+      </c>
+      <c r="G481" t="inlineStr">
+        <is>
+          <t>Junior Level(1-3 years)</t>
+        </is>
+      </c>
+      <c r="H481" t="inlineStr">
+        <is>
+          <t>Full time</t>
+        </is>
+      </c>
+      <c r="I481" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="L481" t="inlineStr">
+        <is>
+          <t>Active listening; problem solving skill; Communication &amp; Negotiation; Customer-oriented with a positive service mindset.</t>
+        </is>
+      </c>
+      <c r="O481" t="inlineStr">
+        <is>
+          <t>October 10th, 2026</t>
+        </is>
+      </c>
+      <c r="P481" t="inlineStr">
+        <is>
+          <t>To Apply Use this Link</t>
+        </is>
+      </c>
+      <c r="Q481" t="inlineStr">
+        <is>
+          <t>https://ethiojobs.net/job/WAhlweiNIf-junior-customer-experience-officer</t>
+        </is>
+      </c>
+      <c r="R481" t="inlineStr">
+        <is>
+          <t>EthioJobs</t>
+        </is>
+      </c>
+      <c r="S481" t="inlineStr">
+        <is>
+          <t>a day ago by</t>
+        </is>
+      </c>
+      <c r="T481" t="inlineStr">
+        <is>
+          <t>2026-09-27 11:02:49 UTC</t>
+        </is>
+      </c>
+      <c r="U481" t="inlineStr">
+        <is>
+          <t>dom_render</t>
+        </is>
+      </c>
+    </row>
+    <row r="482">
+      <c r="A482" t="inlineStr">
+        <is>
+          <t>lhSLqpqXZO</t>
+        </is>
+      </c>
+      <c r="B482" t="inlineStr">
+        <is>
+          <t>Assembly Technician</t>
+        </is>
+      </c>
+      <c r="C482" t="inlineStr">
+        <is>
+          <t>DODAI MANUFACTURING PLC.</t>
+        </is>
+      </c>
+      <c r="D482" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="E482" t="inlineStr">
+        <is>
+          <t>Addis Ababa</t>
+        </is>
+      </c>
+      <c r="F482" t="inlineStr">
+        <is>
+          <t>Office</t>
+        </is>
+      </c>
+      <c r="G482" t="inlineStr">
+        <is>
+          <t>Mid Level(3-5 years)</t>
+        </is>
+      </c>
+      <c r="H482" t="inlineStr">
+        <is>
+          <t>Full time</t>
+        </is>
+      </c>
+      <c r="I482" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="L482" t="inlineStr">
+        <is>
+          <t>Attention to detail; Technical proficiency; analytical, and problem-solving skills</t>
+        </is>
+      </c>
+      <c r="O482" t="inlineStr">
+        <is>
+          <t>October 10th, 2026</t>
+        </is>
+      </c>
+      <c r="P482" t="inlineStr">
+        <is>
+          <t>To apply use this link</t>
+        </is>
+      </c>
+      <c r="Q482" t="inlineStr">
+        <is>
+          <t>https://ethiojobs.net/job/lhSLqpqXZO-assembly-technician</t>
+        </is>
+      </c>
+      <c r="R482" t="inlineStr">
+        <is>
+          <t>EthioJobs</t>
+        </is>
+      </c>
+      <c r="S482" t="inlineStr">
+        <is>
+          <t>a day ago by</t>
+        </is>
+      </c>
+      <c r="T482" t="inlineStr">
+        <is>
+          <t>2026-09-27 11:02:53 UTC</t>
+        </is>
+      </c>
+      <c r="U482" t="inlineStr">
+        <is>
+          <t>dom_render</t>
+        </is>
+      </c>
+    </row>
+    <row r="483">
+      <c r="A483" t="inlineStr">
+        <is>
+          <t>S0kX4KyMd8</t>
+        </is>
+      </c>
+      <c r="B483" t="inlineStr">
+        <is>
+          <t>Intern</t>
+        </is>
+      </c>
+      <c r="C483" t="inlineStr">
+        <is>
+          <t>DODAI MANUFACTURING PLC.</t>
+        </is>
+      </c>
+      <c r="D483" t="inlineStr">
+        <is>
+          <t>Accounting and Finance; Customer Service; Logistics, Transport an...; Engineering</t>
+        </is>
+      </c>
+      <c r="E483" t="inlineStr">
+        <is>
+          <t>Addis Ababa</t>
+        </is>
+      </c>
+      <c r="F483" t="inlineStr">
+        <is>
+          <t>Office</t>
+        </is>
+      </c>
+      <c r="G483" t="inlineStr">
+        <is>
+          <t>Entry Level (Fresh Graduate)</t>
+        </is>
+      </c>
+      <c r="H483" t="inlineStr">
+        <is>
+          <t>Internship</t>
+        </is>
+      </c>
+      <c r="I483" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="J483" t="inlineStr">
+        <is>
+          <t>al Background Requirements</t>
+        </is>
+      </c>
+      <c r="L483" t="inlineStr">
+        <is>
+          <t>Communication; Attention to detail; Excellent analytical, problem-solving, and reporting skills.</t>
+        </is>
+      </c>
+      <c r="O483" t="inlineStr">
+        <is>
+          <t>October 10th, 2026</t>
+        </is>
+      </c>
+      <c r="P483" t="inlineStr">
+        <is>
+          <t>To apply you this link</t>
+        </is>
+      </c>
+      <c r="Q483" t="inlineStr">
+        <is>
+          <t>https://ethiojobs.net/job/S0kX4KyMd8-intern</t>
+        </is>
+      </c>
+      <c r="R483" t="inlineStr">
+        <is>
+          <t>EthioJobs</t>
+        </is>
+      </c>
+      <c r="S483" t="inlineStr">
+        <is>
+          <t>a day ago by</t>
+        </is>
+      </c>
+      <c r="T483" t="inlineStr">
+        <is>
+          <t>2026-09-27 11:02:56 UTC</t>
+        </is>
+      </c>
+      <c r="U483" t="inlineStr">
+        <is>
+          <t>dom_render</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:U1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -45677,7 +46296,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -45747,6 +46366,19 @@
       </c>
       <c r="C5" t="n">
         <v>475</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-09-27 11:02:58 UTC</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>7</v>
+      </c>
+      <c r="C6" t="n">
+        <v>482</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily EthioJobs update 2026-09-28
</commit_message>
<xml_diff>
--- a/ethiojobs_tracker.xlsx
+++ b/ethiojobs_tracker.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U541"/>
+  <dimension ref="A1:U569"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -51748,6 +51748,2629 @@
         </is>
       </c>
     </row>
+    <row r="542">
+      <c r="A542" t="inlineStr">
+        <is>
+          <t>3bUtqNg9OI</t>
+        </is>
+      </c>
+      <c r="B542" t="inlineStr">
+        <is>
+          <t>IT Auditor</t>
+        </is>
+      </c>
+      <c r="C542" t="inlineStr">
+        <is>
+          <t>AMHARA BANK S.C.</t>
+        </is>
+      </c>
+      <c r="D542" t="inlineStr">
+        <is>
+          <t>IT, Computer Science an...; Telecommunications</t>
+        </is>
+      </c>
+      <c r="E542" t="inlineStr">
+        <is>
+          <t>Addis Ababa</t>
+        </is>
+      </c>
+      <c r="F542" t="inlineStr">
+        <is>
+          <t>Office</t>
+        </is>
+      </c>
+      <c r="G542" t="inlineStr">
+        <is>
+          <t>Mid Level(3-5 years)</t>
+        </is>
+      </c>
+      <c r="H542" t="inlineStr">
+        <is>
+          <t>Full time</t>
+        </is>
+      </c>
+      <c r="I542" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="L542" t="inlineStr">
+        <is>
+          <t>Auditing skills; Audit &amp; Compliance Management; Audit Coordination; Audit Documentation; Audit Reporting</t>
+        </is>
+      </c>
+      <c r="O542" t="inlineStr">
+        <is>
+          <t>October 2nd, 2026</t>
+        </is>
+      </c>
+      <c r="P542" t="inlineStr">
+        <is>
+          <t>NB:
+Female applicants highly encouraged
+Only shortlisted candidates will be communicated
+Hard copy or physical applications will not be accepted
+The Bank has the right to cancel the post advertised
+Interested applicants fulfilling the above requirements are invited to apply within five (5) Consecutive days from September 28, 2026to October 02, 2026.
+https://vacancy.amharabank.com.et/.</t>
+        </is>
+      </c>
+      <c r="Q542" t="inlineStr">
+        <is>
+          <t>https://ethiojobs.net/job/3bUtqNg9OI-it-auditor</t>
+        </is>
+      </c>
+      <c r="R542" t="inlineStr">
+        <is>
+          <t>EthioJobs</t>
+        </is>
+      </c>
+      <c r="S542" t="inlineStr">
+        <is>
+          <t>10 minutes ago by</t>
+        </is>
+      </c>
+      <c r="T542" t="inlineStr">
+        <is>
+          <t>2026-09-28 15:31:33 UTC</t>
+        </is>
+      </c>
+      <c r="U542" t="inlineStr">
+        <is>
+          <t>dom_render</t>
+        </is>
+      </c>
+    </row>
+    <row r="543">
+      <c r="A543" t="inlineStr">
+        <is>
+          <t>lVcLdxQAGQ</t>
+        </is>
+      </c>
+      <c r="B543" t="inlineStr">
+        <is>
+          <t>Senior IT Auditor (Re-advertised)</t>
+        </is>
+      </c>
+      <c r="C543" t="inlineStr">
+        <is>
+          <t>AMHARA BANK S.C.</t>
+        </is>
+      </c>
+      <c r="D543" t="inlineStr">
+        <is>
+          <t>Customer Service; IT, Computer Science an...</t>
+        </is>
+      </c>
+      <c r="E543" t="inlineStr">
+        <is>
+          <t>Addis Ababa</t>
+        </is>
+      </c>
+      <c r="F543" t="inlineStr">
+        <is>
+          <t>Office</t>
+        </is>
+      </c>
+      <c r="G543" t="inlineStr">
+        <is>
+          <t>Senior(5-8 years)</t>
+        </is>
+      </c>
+      <c r="H543" t="inlineStr">
+        <is>
+          <t>Full time</t>
+        </is>
+      </c>
+      <c r="I543" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="L543" t="inlineStr">
+        <is>
+          <t>Auditing skills; Audit &amp; Compliance Management; Audit Coordination; Audit Documentation; Audit Reporting</t>
+        </is>
+      </c>
+      <c r="O543" t="inlineStr">
+        <is>
+          <t>October 2nd, 2026</t>
+        </is>
+      </c>
+      <c r="P543" t="inlineStr">
+        <is>
+          <t>NB:
+Female applicants highly encouraged
+Only shortlisted candidates will be communicated
+Hard copy or physical applications will not be accepted
+The Bank has the right to cancel the post advertised
+Interested applicants fulfilling the above requirements are invited to apply within five (5) Consecutive days from September 28, 2026to October 02, 2026.
+https://vacancy.amharabank.com.et/.</t>
+        </is>
+      </c>
+      <c r="Q543" t="inlineStr">
+        <is>
+          <t>https://ethiojobs.net/job/lVcLdxQAGQ-senior-it-auditor-re-advertised</t>
+        </is>
+      </c>
+      <c r="R543" t="inlineStr">
+        <is>
+          <t>EthioJobs</t>
+        </is>
+      </c>
+      <c r="S543" t="inlineStr">
+        <is>
+          <t>20 minutes ago by</t>
+        </is>
+      </c>
+      <c r="T543" t="inlineStr">
+        <is>
+          <t>2026-09-28 15:31:36 UTC</t>
+        </is>
+      </c>
+      <c r="U543" t="inlineStr">
+        <is>
+          <t>dom_render</t>
+        </is>
+      </c>
+    </row>
+    <row r="544">
+      <c r="A544" t="inlineStr">
+        <is>
+          <t>YdnWUnjVPz</t>
+        </is>
+      </c>
+      <c r="B544" t="inlineStr">
+        <is>
+          <t>Senior Service Quality Assurance Officer</t>
+        </is>
+      </c>
+      <c r="C544" t="inlineStr">
+        <is>
+          <t>AMHARA BANK S.C.</t>
+        </is>
+      </c>
+      <c r="D544" t="inlineStr">
+        <is>
+          <t>Accounting and Finance; Banking and Insurance; Business and Administra...; Economics</t>
+        </is>
+      </c>
+      <c r="E544" t="inlineStr">
+        <is>
+          <t>Addis Ababa</t>
+        </is>
+      </c>
+      <c r="F544" t="inlineStr">
+        <is>
+          <t>Office</t>
+        </is>
+      </c>
+      <c r="G544" t="inlineStr">
+        <is>
+          <t>Senior(5-8 years)</t>
+        </is>
+      </c>
+      <c r="H544" t="inlineStr">
+        <is>
+          <t>Full time</t>
+        </is>
+      </c>
+      <c r="I544" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="L544" t="inlineStr">
+        <is>
+          <t>Quality control; Quality assurance; Quality assurance and compliance focus</t>
+        </is>
+      </c>
+      <c r="O544" t="inlineStr">
+        <is>
+          <t>October 2nd, 2026</t>
+        </is>
+      </c>
+      <c r="P544" t="inlineStr">
+        <is>
+          <t>NB:
+Female applicants highly encouraged
+Only shortlisted candidates will be communicated
+Hard copy or physical applications will not be accepted
+The Bank has the right to cancel the post advertised
+Interested applicants fulfilling the above requirements are invited to apply within five (5) Consecutive days from September 28, 2026to October 02, 2026.
+https://vacancy.amharabank.com.et/.</t>
+        </is>
+      </c>
+      <c r="Q544" t="inlineStr">
+        <is>
+          <t>https://ethiojobs.net/job/YdnWUnjVPz-senior-service-quality-assurance-officer</t>
+        </is>
+      </c>
+      <c r="R544" t="inlineStr">
+        <is>
+          <t>EthioJobs</t>
+        </is>
+      </c>
+      <c r="S544" t="inlineStr">
+        <is>
+          <t>20 minutes ago by</t>
+        </is>
+      </c>
+      <c r="T544" t="inlineStr">
+        <is>
+          <t>2026-09-28 15:31:39 UTC</t>
+        </is>
+      </c>
+      <c r="U544" t="inlineStr">
+        <is>
+          <t>dom_render</t>
+        </is>
+      </c>
+    </row>
+    <row r="545">
+      <c r="A545" t="inlineStr">
+        <is>
+          <t>1zXFys9G3H</t>
+        </is>
+      </c>
+      <c r="B545" t="inlineStr">
+        <is>
+          <t>Financial Management Systems Expert</t>
+        </is>
+      </c>
+      <c r="C545" t="inlineStr">
+        <is>
+          <t>NATIONAL ELECTION BOARD OF ETHIOPIA(NEBE)</t>
+        </is>
+      </c>
+      <c r="D545" t="inlineStr">
+        <is>
+          <t>Accounting and Finance</t>
+        </is>
+      </c>
+      <c r="E545" t="inlineStr">
+        <is>
+          <t>Addis Ababa</t>
+        </is>
+      </c>
+      <c r="F545" t="inlineStr">
+        <is>
+          <t>Office</t>
+        </is>
+      </c>
+      <c r="G545" t="inlineStr">
+        <is>
+          <t>Senior(5-8 years)</t>
+        </is>
+      </c>
+      <c r="H545" t="inlineStr">
+        <is>
+          <t>Full time</t>
+        </is>
+      </c>
+      <c r="I545" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J545" t="inlineStr">
+        <is>
+          <t>and</t>
+        </is>
+      </c>
+      <c r="K545" t="inlineStr">
+        <is>
+          <t>5 years</t>
+        </is>
+      </c>
+      <c r="L545" t="inlineStr">
+        <is>
+          <t>Financial planning; Accounting; xperience and knowledge of IFMIS, IFRIS is required</t>
+        </is>
+      </c>
+      <c r="O545" t="inlineStr">
+        <is>
+          <t>October 8th, 2026</t>
+        </is>
+      </c>
+      <c r="P545" t="inlineStr">
+        <is>
+          <t>INTERESTED APPLICANTS ARE INVITED TO SEND NON-RETURNABLE:
+Application letter that explains why you fit for the post and updated CV, and Three work related referees;
+Application letter &amp; resume should be saved by full name of Applicants.
+Only short-listed candidates will be contacted for further screening.
+Those who are interested can only apply through the attached link               
+https://nebe-election.org/apply  within 10 days from this announcement.
+Female candidates are encouraged to apply!</t>
+        </is>
+      </c>
+      <c r="Q545" t="inlineStr">
+        <is>
+          <t>https://ethiojobs.net/job/1zXFys9G3H-financial-management-systems-expert</t>
+        </is>
+      </c>
+      <c r="R545" t="inlineStr">
+        <is>
+          <t>EthioJobs</t>
+        </is>
+      </c>
+      <c r="S545" t="inlineStr">
+        <is>
+          <t>an hour ago by</t>
+        </is>
+      </c>
+      <c r="T545" t="inlineStr">
+        <is>
+          <t>2026-09-28 15:31:42 UTC</t>
+        </is>
+      </c>
+      <c r="U545" t="inlineStr">
+        <is>
+          <t>dom_render</t>
+        </is>
+      </c>
+    </row>
+    <row r="546">
+      <c r="A546" t="inlineStr">
+        <is>
+          <t>JkNAt5FtQR</t>
+        </is>
+      </c>
+      <c r="B546" t="inlineStr">
+        <is>
+          <t>Junior Budget Expert I</t>
+        </is>
+      </c>
+      <c r="C546" t="inlineStr">
+        <is>
+          <t>NATIONAL ELECTION BOARD OF ETHIOPIA(NEBE)</t>
+        </is>
+      </c>
+      <c r="D546" t="inlineStr">
+        <is>
+          <t>Accounting and Finance</t>
+        </is>
+      </c>
+      <c r="E546" t="inlineStr">
+        <is>
+          <t>Addis Ababa</t>
+        </is>
+      </c>
+      <c r="F546" t="inlineStr">
+        <is>
+          <t>Office</t>
+        </is>
+      </c>
+      <c r="G546" t="inlineStr">
+        <is>
+          <t>Junior Level(1-3 years)</t>
+        </is>
+      </c>
+      <c r="H546" t="inlineStr">
+        <is>
+          <t>Full time</t>
+        </is>
+      </c>
+      <c r="I546" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J546" t="inlineStr">
+        <is>
+          <t>and</t>
+        </is>
+      </c>
+      <c r="K546" t="inlineStr">
+        <is>
+          <t>0 years</t>
+        </is>
+      </c>
+      <c r="L546" t="inlineStr">
+        <is>
+          <t>Communication; Attention to detail; Budgeting</t>
+        </is>
+      </c>
+      <c r="O546" t="inlineStr">
+        <is>
+          <t>October 8th, 2026</t>
+        </is>
+      </c>
+      <c r="P546" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      INTERESTED APPLICANTS ARE INVITED TO SEND NON-RETURNABLE:
+Application letter that explains why you fit for the post and updated CV, and Three work related referees;
+Application letter &amp; resume should be saved by full name of Applicants.
+Only short-listed candidates will be contacted for further screening.
+Those who are interested can only apply through the attached link               
+https://nebe-election.org/apply within 10 days from this announcement.
+Female candidates are encouraged to apply!</t>
+        </is>
+      </c>
+      <c r="Q546" t="inlineStr">
+        <is>
+          <t>https://ethiojobs.net/job/JkNAt5FtQR-junior-budget-expert-i</t>
+        </is>
+      </c>
+      <c r="R546" t="inlineStr">
+        <is>
+          <t>EthioJobs</t>
+        </is>
+      </c>
+      <c r="S546" t="inlineStr">
+        <is>
+          <t>an hour ago by</t>
+        </is>
+      </c>
+      <c r="T546" t="inlineStr">
+        <is>
+          <t>2026-09-28 15:31:45 UTC</t>
+        </is>
+      </c>
+      <c r="U546" t="inlineStr">
+        <is>
+          <t>dom_render</t>
+        </is>
+      </c>
+    </row>
+    <row r="547">
+      <c r="A547" t="inlineStr">
+        <is>
+          <t>XBIqNMTnRU</t>
+        </is>
+      </c>
+      <c r="B547" t="inlineStr">
+        <is>
+          <t>Graduate in Training (GIT) - Sales</t>
+        </is>
+      </c>
+      <c r="C547" t="inlineStr">
+        <is>
+          <t>HABESHA BREWERIES SC.</t>
+        </is>
+      </c>
+      <c r="D547" t="inlineStr">
+        <is>
+          <t>Sales and Marketing</t>
+        </is>
+      </c>
+      <c r="E547" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="F547" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="G547" t="inlineStr">
+        <is>
+          <t>Junior Level(1-3 years)</t>
+        </is>
+      </c>
+      <c r="H547" t="inlineStr">
+        <is>
+          <t>Full time</t>
+        </is>
+      </c>
+      <c r="I547" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="J547" t="inlineStr">
+        <is>
+          <t>Bachelor's degree</t>
+        </is>
+      </c>
+      <c r="L547" t="inlineStr">
+        <is>
+          <t>Continuous learning; Result Driven; customer communication and understanding capabilities; Teamwork and collaboration; action driven</t>
+        </is>
+      </c>
+      <c r="N547" t="inlineStr">
+        <is>
+          <t>,</t>
+        </is>
+      </c>
+      <c r="O547" t="inlineStr">
+        <is>
+          <t>October 10th, 2026</t>
+        </is>
+      </c>
+      <c r="P547" t="inlineStr">
+        <is>
+          <t>Interested candidates who meet the above criteria should submit their updated CV and academic transcripts by October 10, 2028.
+Application Tip: While not a strict requirement, candidates are highly encouraged to detail any extracurricular achievements, club roles, or volunteer experience in their CV or cover letter to maximize their chances.
+Habesha Breweries is an Equal Opportunity Employer. Only shortlisted candidates will be contacted for the assessment phase.</t>
+        </is>
+      </c>
+      <c r="Q547" t="inlineStr">
+        <is>
+          <t>https://ethiojobs.net/job/XBIqNMTnRU-graduate-in-training-git-sales</t>
+        </is>
+      </c>
+      <c r="R547" t="inlineStr">
+        <is>
+          <t>EthioJobs</t>
+        </is>
+      </c>
+      <c r="S547" t="inlineStr">
+        <is>
+          <t>an hour ago by</t>
+        </is>
+      </c>
+      <c r="T547" t="inlineStr">
+        <is>
+          <t>2026-09-28 15:31:48 UTC</t>
+        </is>
+      </c>
+      <c r="U547" t="inlineStr">
+        <is>
+          <t>dom_render</t>
+        </is>
+      </c>
+    </row>
+    <row r="548">
+      <c r="A548" t="inlineStr">
+        <is>
+          <t>Ddyortlph0</t>
+        </is>
+      </c>
+      <c r="B548" t="inlineStr">
+        <is>
+          <t>Technology Product Manager</t>
+        </is>
+      </c>
+      <c r="C548" t="inlineStr">
+        <is>
+          <t>AMERICAN COLLEGE OF TECHNOLOGY (ACT)</t>
+        </is>
+      </c>
+      <c r="D548" t="inlineStr">
+        <is>
+          <t>Technology; Development and Project...</t>
+        </is>
+      </c>
+      <c r="E548" t="inlineStr">
+        <is>
+          <t>Addis Ababa</t>
+        </is>
+      </c>
+      <c r="F548" t="inlineStr">
+        <is>
+          <t>Office</t>
+        </is>
+      </c>
+      <c r="G548" t="inlineStr">
+        <is>
+          <t>Junior Level(1-3 years)</t>
+        </is>
+      </c>
+      <c r="H548" t="inlineStr">
+        <is>
+          <t>Full time</t>
+        </is>
+      </c>
+      <c r="I548" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K548" t="inlineStr">
+        <is>
+          <t>1-3 years</t>
+        </is>
+      </c>
+      <c r="L548" t="inlineStr">
+        <is>
+          <t>Good knowledge of manufacturing systems, ERP tools (SAP), and digital production platforms.; Ability to support Resident Engineer in technical and administrative tasks; Computer Science, Information System, Information Technology, Computer Engineering; Computer Science, Software Engineering, Information Technology; Desired Skill; Product knowledge; Good knowledge of manufacturing systems, ERP tools (SAP), and digital production platforms.; Computer Science, Information System, Information Technology, Computer Engineering; Computer Science, Software Engineering, Information Technology</t>
+        </is>
+      </c>
+      <c r="O548" t="inlineStr">
+        <is>
+          <t>October 17th, 2026</t>
+        </is>
+      </c>
+      <c r="P548" t="inlineStr">
+        <is>
+          <t>Interested and qualified applicants should submit their CV, cover letter, and copies of academic credentials via website actjobs</t>
+        </is>
+      </c>
+      <c r="Q548" t="inlineStr">
+        <is>
+          <t>https://ethiojobs.net/job/Ddyortlph0-technology-product-manager</t>
+        </is>
+      </c>
+      <c r="R548" t="inlineStr">
+        <is>
+          <t>EthioJobs</t>
+        </is>
+      </c>
+      <c r="S548" t="inlineStr">
+        <is>
+          <t>an hour ago by</t>
+        </is>
+      </c>
+      <c r="T548" t="inlineStr">
+        <is>
+          <t>2026-09-28 15:31:51 UTC</t>
+        </is>
+      </c>
+      <c r="U548" t="inlineStr">
+        <is>
+          <t>dom_render</t>
+        </is>
+      </c>
+    </row>
+    <row r="549">
+      <c r="A549" t="inlineStr">
+        <is>
+          <t>TEA3tPEr88</t>
+        </is>
+      </c>
+      <c r="B549" t="inlineStr">
+        <is>
+          <t>Senior Finance Expert</t>
+        </is>
+      </c>
+      <c r="C549" t="inlineStr">
+        <is>
+          <t>NATIONAL ELECTION BOARD OF ETHIOPIA(NEBE)</t>
+        </is>
+      </c>
+      <c r="D549" t="inlineStr">
+        <is>
+          <t>Accounting and Finance</t>
+        </is>
+      </c>
+      <c r="E549" t="inlineStr">
+        <is>
+          <t>Addis Ababa</t>
+        </is>
+      </c>
+      <c r="F549" t="inlineStr">
+        <is>
+          <t>Office</t>
+        </is>
+      </c>
+      <c r="G549" t="inlineStr">
+        <is>
+          <t>Senior(5-8 years)</t>
+        </is>
+      </c>
+      <c r="H549" t="inlineStr">
+        <is>
+          <t>Full time</t>
+        </is>
+      </c>
+      <c r="I549" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J549" t="inlineStr">
+        <is>
+          <t>and</t>
+        </is>
+      </c>
+      <c r="K549" t="inlineStr">
+        <is>
+          <t>7 years</t>
+        </is>
+      </c>
+      <c r="L549" t="inlineStr">
+        <is>
+          <t>Accounting; Accounting Principles (GAAP), IFRS and ERP; xperience and knowledge of IFMIS, IFRIS is required; Accounts Payable &amp; Receivable</t>
+        </is>
+      </c>
+      <c r="O549" t="inlineStr">
+        <is>
+          <t>October 8th, 2026</t>
+        </is>
+      </c>
+      <c r="P549" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      INTERESTED APPLICANTS ARE INVITED TO SEND NON-RETURNABLE:
+Application letter that explains why you fit for the post and updated CV, and Three work related referees;
+Application letter &amp; resume should be saved by full name of Applicants.
+Only short-listed candidates will be contacted for further screening.
+Those who are interested can only apply through the attached link
+https://nebe-election.org/apply  Within 10 days from this announcement.
+Female candidates are encouraged to apply!</t>
+        </is>
+      </c>
+      <c r="Q549" t="inlineStr">
+        <is>
+          <t>https://ethiojobs.net/job/TEA3tPEr88-senior-finance-expert</t>
+        </is>
+      </c>
+      <c r="R549" t="inlineStr">
+        <is>
+          <t>EthioJobs</t>
+        </is>
+      </c>
+      <c r="S549" t="inlineStr">
+        <is>
+          <t>2 hours ago by</t>
+        </is>
+      </c>
+      <c r="T549" t="inlineStr">
+        <is>
+          <t>2026-09-28 15:31:54 UTC</t>
+        </is>
+      </c>
+      <c r="U549" t="inlineStr">
+        <is>
+          <t>dom_render</t>
+        </is>
+      </c>
+    </row>
+    <row r="550">
+      <c r="A550" t="inlineStr">
+        <is>
+          <t>NXN8XMleIi</t>
+        </is>
+      </c>
+      <c r="B550" t="inlineStr">
+        <is>
+          <t>Head of Student Affairs</t>
+        </is>
+      </c>
+      <c r="C550" t="inlineStr">
+        <is>
+          <t>AMERICAN COLLEGE OF TECHNOLOGY (ACT)</t>
+        </is>
+      </c>
+      <c r="D550" t="inlineStr">
+        <is>
+          <t>Management</t>
+        </is>
+      </c>
+      <c r="E550" t="inlineStr">
+        <is>
+          <t>Addis Ababa</t>
+        </is>
+      </c>
+      <c r="F550" t="inlineStr">
+        <is>
+          <t>Office</t>
+        </is>
+      </c>
+      <c r="G550" t="inlineStr">
+        <is>
+          <t>Junior Level(1-3 years)</t>
+        </is>
+      </c>
+      <c r="H550" t="inlineStr">
+        <is>
+          <t>Full time</t>
+        </is>
+      </c>
+      <c r="I550" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K550" t="inlineStr">
+        <is>
+          <t>1-3 years</t>
+        </is>
+      </c>
+      <c r="L550" t="inlineStr">
+        <is>
+          <t>Conflict Resolution; A genuine passion for education and student development.; Youth development, Sport management, Physical education; Desired Skill; Analytical thinking and problem-solving skills.; analytical, and problem-solving skills; Analytical and problem-solving skills; Analytical: strong problem-solving and analytical abilities.</t>
+        </is>
+      </c>
+      <c r="O550" t="inlineStr">
+        <is>
+          <t>October 17th, 2026</t>
+        </is>
+      </c>
+      <c r="P550" t="inlineStr">
+        <is>
+          <t>Interested and qualified applicants should submit their CV, cover letter, and copies of academic credentials via website actjobs</t>
+        </is>
+      </c>
+      <c r="Q550" t="inlineStr">
+        <is>
+          <t>https://ethiojobs.net/job/NXN8XMleIi-head-of-student-affairs</t>
+        </is>
+      </c>
+      <c r="R550" t="inlineStr">
+        <is>
+          <t>EthioJobs</t>
+        </is>
+      </c>
+      <c r="S550" t="inlineStr">
+        <is>
+          <t>2 hours ago by</t>
+        </is>
+      </c>
+      <c r="T550" t="inlineStr">
+        <is>
+          <t>2026-09-28 15:31:57 UTC</t>
+        </is>
+      </c>
+      <c r="U550" t="inlineStr">
+        <is>
+          <t>dom_render</t>
+        </is>
+      </c>
+    </row>
+    <row r="551">
+      <c r="A551" t="inlineStr">
+        <is>
+          <t>ZN8rd4UfEs</t>
+        </is>
+      </c>
+      <c r="B551" t="inlineStr">
+        <is>
+          <t>Finance Expert</t>
+        </is>
+      </c>
+      <c r="C551" t="inlineStr">
+        <is>
+          <t>NATIONAL ELECTION BOARD OF ETHIOPIA(NEBE)</t>
+        </is>
+      </c>
+      <c r="D551" t="inlineStr">
+        <is>
+          <t>Accounting and Finance</t>
+        </is>
+      </c>
+      <c r="E551" t="inlineStr">
+        <is>
+          <t>Addis Ababa</t>
+        </is>
+      </c>
+      <c r="F551" t="inlineStr">
+        <is>
+          <t>Office</t>
+        </is>
+      </c>
+      <c r="G551" t="inlineStr">
+        <is>
+          <t>Senior(5-8 years)</t>
+        </is>
+      </c>
+      <c r="H551" t="inlineStr">
+        <is>
+          <t>Full time</t>
+        </is>
+      </c>
+      <c r="I551" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J551" t="inlineStr">
+        <is>
+          <t>and</t>
+        </is>
+      </c>
+      <c r="K551" t="inlineStr">
+        <is>
+          <t>5 years</t>
+        </is>
+      </c>
+      <c r="L551" t="inlineStr">
+        <is>
+          <t>Accounting; Accounting Principles (GAAP), IFRS and ERP; xperience and knowledge of IFMIS, IFRIS is required</t>
+        </is>
+      </c>
+      <c r="O551" t="inlineStr">
+        <is>
+          <t>October 8th, 2026</t>
+        </is>
+      </c>
+      <c r="P551" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      INTERESTED APPLICANTS ARE INVITED TO SEND NON-RETURNABLE:
+Application letter that explains why you fit for the post and updated CV, and Three work related referees;
+Application letter &amp; resume should be saved by full name of Applicants.
+Only short-listed candidates will be contacted for further screening.
+Those who are interested can only apply through the attached link
+https://nebe-election.org/apply  Within 10 days from this announcement.
+Female candidates are encouraged to apply!</t>
+        </is>
+      </c>
+      <c r="Q551" t="inlineStr">
+        <is>
+          <t>https://ethiojobs.net/job/ZN8rd4UfEs-finance-expert</t>
+        </is>
+      </c>
+      <c r="R551" t="inlineStr">
+        <is>
+          <t>EthioJobs</t>
+        </is>
+      </c>
+      <c r="S551" t="inlineStr">
+        <is>
+          <t>2 hours ago by</t>
+        </is>
+      </c>
+      <c r="T551" t="inlineStr">
+        <is>
+          <t>2026-09-28 15:32:00 UTC</t>
+        </is>
+      </c>
+      <c r="U551" t="inlineStr">
+        <is>
+          <t>dom_render</t>
+        </is>
+      </c>
+    </row>
+    <row r="552">
+      <c r="A552" t="inlineStr">
+        <is>
+          <t>TU2FZxc1NN</t>
+        </is>
+      </c>
+      <c r="B552" t="inlineStr">
+        <is>
+          <t>SENIOR ACCOUNTANT</t>
+        </is>
+      </c>
+      <c r="C552" t="inlineStr">
+        <is>
+          <t>SAM BUSINESS GROUP</t>
+        </is>
+      </c>
+      <c r="D552" t="inlineStr">
+        <is>
+          <t>Accounting and Finance</t>
+        </is>
+      </c>
+      <c r="E552" t="inlineStr">
+        <is>
+          <t>Addis Ababa</t>
+        </is>
+      </c>
+      <c r="F552" t="inlineStr">
+        <is>
+          <t>Office</t>
+        </is>
+      </c>
+      <c r="G552" t="inlineStr">
+        <is>
+          <t>Executive(VP, Director)</t>
+        </is>
+      </c>
+      <c r="H552" t="inlineStr">
+        <is>
+          <t>Full time</t>
+        </is>
+      </c>
+      <c r="I552" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K552" t="inlineStr">
+        <is>
+          <t>8-12 years</t>
+        </is>
+      </c>
+      <c r="L552" t="inlineStr">
+        <is>
+          <t>Adaptability; Accounting; Desired Skill; Communication</t>
+        </is>
+      </c>
+      <c r="N552" t="inlineStr">
+        <is>
+          <t>45,000</t>
+        </is>
+      </c>
+      <c r="O552" t="inlineStr">
+        <is>
+          <t>October 29th, 2026</t>
+        </is>
+      </c>
+      <c r="P552" t="inlineStr">
+        <is>
+          <t>All candidates can apply through telegram or WhatsApp
++251 91 151 6723
+@Eyouel_S</t>
+        </is>
+      </c>
+      <c r="Q552" t="inlineStr">
+        <is>
+          <t>https://ethiojobs.net/job/TU2FZxc1NN-senior-accountant</t>
+        </is>
+      </c>
+      <c r="R552" t="inlineStr">
+        <is>
+          <t>EthioJobs</t>
+        </is>
+      </c>
+      <c r="S552" t="inlineStr">
+        <is>
+          <t>2 hours ago by</t>
+        </is>
+      </c>
+      <c r="T552" t="inlineStr">
+        <is>
+          <t>2026-09-28 15:32:03 UTC</t>
+        </is>
+      </c>
+      <c r="U552" t="inlineStr">
+        <is>
+          <t>dom_render</t>
+        </is>
+      </c>
+    </row>
+    <row r="553">
+      <c r="A553" t="inlineStr">
+        <is>
+          <t>zY3zAQ03Jp</t>
+        </is>
+      </c>
+      <c r="B553" t="inlineStr">
+        <is>
+          <t>Electro-Mechanical Technician</t>
+        </is>
+      </c>
+      <c r="C553" t="inlineStr">
+        <is>
+          <t>SCEPTO IMPORT</t>
+        </is>
+      </c>
+      <c r="D553" t="inlineStr">
+        <is>
+          <t>Engineering; Natural Sciences; Social Sciences and Com...</t>
+        </is>
+      </c>
+      <c r="E553" t="inlineStr">
+        <is>
+          <t>Addis Ababa</t>
+        </is>
+      </c>
+      <c r="F553" t="inlineStr">
+        <is>
+          <t>Office</t>
+        </is>
+      </c>
+      <c r="G553" t="inlineStr">
+        <is>
+          <t>Mid Level(3-5 years)</t>
+        </is>
+      </c>
+      <c r="H553" t="inlineStr">
+        <is>
+          <t>Full time</t>
+        </is>
+      </c>
+      <c r="I553" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J553" t="inlineStr">
+        <is>
+          <t>Diploma</t>
+        </is>
+      </c>
+      <c r="L553" t="inlineStr">
+        <is>
+          <t>Communication</t>
+        </is>
+      </c>
+      <c r="O553" t="inlineStr">
+        <is>
+          <t>October 29th, 2026</t>
+        </is>
+      </c>
+      <c r="P553" t="inlineStr">
+        <is>
+          <t>Interested and qualified candidates are invited to submit your CV and relevant credentials to:
+SCEPTO IMPORT PLC
+📧 Email: Jobs@scepto.net</t>
+        </is>
+      </c>
+      <c r="Q553" t="inlineStr">
+        <is>
+          <t>https://ethiojobs.net/job/zY3zAQ03Jp-electro-mechanical-technician</t>
+        </is>
+      </c>
+      <c r="R553" t="inlineStr">
+        <is>
+          <t>EthioJobs</t>
+        </is>
+      </c>
+      <c r="S553" t="inlineStr">
+        <is>
+          <t>2 hours ago by</t>
+        </is>
+      </c>
+      <c r="T553" t="inlineStr">
+        <is>
+          <t>2026-09-28 15:32:06 UTC</t>
+        </is>
+      </c>
+      <c r="U553" t="inlineStr">
+        <is>
+          <t>dom_render</t>
+        </is>
+      </c>
+    </row>
+    <row r="554">
+      <c r="A554" t="inlineStr">
+        <is>
+          <t>EXyWvvhJ7Y</t>
+        </is>
+      </c>
+      <c r="B554" t="inlineStr">
+        <is>
+          <t>Senior Officer, Core Systems</t>
+        </is>
+      </c>
+      <c r="C554" t="inlineStr">
+        <is>
+          <t>ZEMEN BANK S.C</t>
+        </is>
+      </c>
+      <c r="D554" t="inlineStr">
+        <is>
+          <t>Banking and Insurance</t>
+        </is>
+      </c>
+      <c r="E554" t="inlineStr">
+        <is>
+          <t>Addis Ababa</t>
+        </is>
+      </c>
+      <c r="F554" t="inlineStr">
+        <is>
+          <t>Office</t>
+        </is>
+      </c>
+      <c r="G554" t="inlineStr">
+        <is>
+          <t>Mid Level(3-5 years)</t>
+        </is>
+      </c>
+      <c r="H554" t="inlineStr">
+        <is>
+          <t>Full time</t>
+        </is>
+      </c>
+      <c r="I554" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J554" t="inlineStr">
+        <is>
+          <t>Bachelor's degree</t>
+        </is>
+      </c>
+      <c r="L554" t="inlineStr">
+        <is>
+          <t>Digital security; Communication; Network administration</t>
+        </is>
+      </c>
+      <c r="O554" t="inlineStr">
+        <is>
+          <t>October 5th, 2026</t>
+        </is>
+      </c>
+      <c r="P554" t="inlineStr">
+        <is>
+          <t>Interested and qualified candidates can apply through www.ethiojobs.net. Please attach your updated CV and credentials in PDF format.
+NB; In person applications are not Acceptable.</t>
+        </is>
+      </c>
+      <c r="Q554" t="inlineStr">
+        <is>
+          <t>https://ethiojobs.net/job/EXyWvvhJ7Y-senior-officer-core-systems</t>
+        </is>
+      </c>
+      <c r="R554" t="inlineStr">
+        <is>
+          <t>EthioJobs</t>
+        </is>
+      </c>
+      <c r="S554" t="inlineStr">
+        <is>
+          <t>2 hours ago by</t>
+        </is>
+      </c>
+      <c r="T554" t="inlineStr">
+        <is>
+          <t>2026-09-28 15:32:09 UTC</t>
+        </is>
+      </c>
+      <c r="U554" t="inlineStr">
+        <is>
+          <t>dom_render</t>
+        </is>
+      </c>
+    </row>
+    <row r="555">
+      <c r="A555" t="inlineStr">
+        <is>
+          <t>HfmOr4zC4u</t>
+        </is>
+      </c>
+      <c r="B555" t="inlineStr">
+        <is>
+          <t>Administrative Officer</t>
+        </is>
+      </c>
+      <c r="C555" t="inlineStr">
+        <is>
+          <t>ETHIOCHICKEN</t>
+        </is>
+      </c>
+      <c r="D555" t="inlineStr">
+        <is>
+          <t>Admin, Secretarial, and...</t>
+        </is>
+      </c>
+      <c r="E555" t="inlineStr">
+        <is>
+          <t>Addis Ababa</t>
+        </is>
+      </c>
+      <c r="F555" t="inlineStr">
+        <is>
+          <t>Office</t>
+        </is>
+      </c>
+      <c r="G555" t="inlineStr">
+        <is>
+          <t>Entry Level (Fresh Graduate)</t>
+        </is>
+      </c>
+      <c r="H555" t="inlineStr">
+        <is>
+          <t>Full time</t>
+        </is>
+      </c>
+      <c r="I555" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J555" t="inlineStr">
+        <is>
+          <t>Bachelor's degree</t>
+        </is>
+      </c>
+      <c r="K555" t="inlineStr">
+        <is>
+          <t>0-1 years</t>
+        </is>
+      </c>
+      <c r="L555" t="inlineStr">
+        <is>
+          <t>Ability to coordinate multiple tasks and work under pressure.; Ability to work under pressure and meet deadlines; Desired Skill; Documentation; Excellent communication and interpersonal abilities.</t>
+        </is>
+      </c>
+      <c r="O555" t="inlineStr">
+        <is>
+          <t>October 5th, 2026</t>
+        </is>
+      </c>
+      <c r="P555" t="inlineStr">
+        <is>
+          <t>APPLICATION INSTRUCTIONS 
+Please title your application with the subject line: - "Administrative Officer”
+Only candidates meeting the required qualifications are invited to send their applications (Cover Letter) including a detailed CV to 
+careers@ethiochicken.com 
+Women are highly encouraged to apply</t>
+        </is>
+      </c>
+      <c r="Q555" t="inlineStr">
+        <is>
+          <t>https://ethiojobs.net/job/HfmOr4zC4u-administrative-officer</t>
+        </is>
+      </c>
+      <c r="R555" t="inlineStr">
+        <is>
+          <t>EthioJobs</t>
+        </is>
+      </c>
+      <c r="S555" t="inlineStr">
+        <is>
+          <t>2 hours ago by</t>
+        </is>
+      </c>
+      <c r="T555" t="inlineStr">
+        <is>
+          <t>2026-09-28 15:32:12 UTC</t>
+        </is>
+      </c>
+      <c r="U555" t="inlineStr">
+        <is>
+          <t>dom_render</t>
+        </is>
+      </c>
+    </row>
+    <row r="556">
+      <c r="A556" t="inlineStr">
+        <is>
+          <t>o7oIUnAxb5</t>
+        </is>
+      </c>
+      <c r="B556" t="inlineStr">
+        <is>
+          <t>Officer, Network Support (Re-Advert)</t>
+        </is>
+      </c>
+      <c r="C556" t="inlineStr">
+        <is>
+          <t>ZEMEN BANK S.C</t>
+        </is>
+      </c>
+      <c r="D556" t="inlineStr">
+        <is>
+          <t>Banking and Insurance</t>
+        </is>
+      </c>
+      <c r="E556" t="inlineStr">
+        <is>
+          <t>Addis Ababa</t>
+        </is>
+      </c>
+      <c r="F556" t="inlineStr">
+        <is>
+          <t>Office</t>
+        </is>
+      </c>
+      <c r="G556" t="inlineStr">
+        <is>
+          <t>Mid Level(3-5 years)</t>
+        </is>
+      </c>
+      <c r="H556" t="inlineStr">
+        <is>
+          <t>Full time</t>
+        </is>
+      </c>
+      <c r="I556" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J556" t="inlineStr">
+        <is>
+          <t>Bachelor's degree</t>
+        </is>
+      </c>
+      <c r="K556" t="inlineStr">
+        <is>
+          <t>3-5 years</t>
+        </is>
+      </c>
+      <c r="L556" t="inlineStr">
+        <is>
+          <t>Cloud networking and file sharing</t>
+        </is>
+      </c>
+      <c r="O556" t="inlineStr">
+        <is>
+          <t>October 5th, 2026</t>
+        </is>
+      </c>
+      <c r="P556" t="inlineStr">
+        <is>
+          <t>Interested and qualified candidates can apply through www.ethiojobs.net. Please attach your updated CV and credentials in PDF format.
+NB; In person applications are not Acceptable.</t>
+        </is>
+      </c>
+      <c r="Q556" t="inlineStr">
+        <is>
+          <t>https://ethiojobs.net/job/o7oIUnAxb5-officer-network-support-re-advert</t>
+        </is>
+      </c>
+      <c r="R556" t="inlineStr">
+        <is>
+          <t>EthioJobs</t>
+        </is>
+      </c>
+      <c r="S556" t="inlineStr">
+        <is>
+          <t>2 hours ago by</t>
+        </is>
+      </c>
+      <c r="T556" t="inlineStr">
+        <is>
+          <t>2026-09-28 15:32:15 UTC</t>
+        </is>
+      </c>
+      <c r="U556" t="inlineStr">
+        <is>
+          <t>dom_render</t>
+        </is>
+      </c>
+    </row>
+    <row r="557">
+      <c r="A557" t="inlineStr">
+        <is>
+          <t>43dTsNxsou</t>
+        </is>
+      </c>
+      <c r="B557" t="inlineStr">
+        <is>
+          <t>CSO III – Accounts (For Ambo &amp; Nekemte Banking Center)</t>
+        </is>
+      </c>
+      <c r="C557" t="inlineStr">
+        <is>
+          <t>ZEMEN BANK S.C</t>
+        </is>
+      </c>
+      <c r="D557" t="inlineStr">
+        <is>
+          <t>Banking and Insurance</t>
+        </is>
+      </c>
+      <c r="E557" t="inlineStr">
+        <is>
+          <t>Oromia</t>
+        </is>
+      </c>
+      <c r="F557" t="inlineStr">
+        <is>
+          <t>Office</t>
+        </is>
+      </c>
+      <c r="O557" t="inlineStr">
+        <is>
+          <t>October 5th, 2026</t>
+        </is>
+      </c>
+      <c r="Q557" t="inlineStr">
+        <is>
+          <t>https://ethiojobs.net/job/43dTsNxsou-cso-iii-accounts-for-ambo-banking-center</t>
+        </is>
+      </c>
+      <c r="R557" t="inlineStr">
+        <is>
+          <t>EthioJobs</t>
+        </is>
+      </c>
+      <c r="S557" t="inlineStr">
+        <is>
+          <t>2 hours ago by</t>
+        </is>
+      </c>
+      <c r="T557" t="inlineStr">
+        <is>
+          <t>2026-09-28 15:32:46 UTC</t>
+        </is>
+      </c>
+      <c r="U557" t="inlineStr">
+        <is>
+          <t>listing_only</t>
+        </is>
+      </c>
+    </row>
+    <row r="558">
+      <c r="A558" t="inlineStr">
+        <is>
+          <t>UYwV987S7G</t>
+        </is>
+      </c>
+      <c r="B558" t="inlineStr">
+        <is>
+          <t>Section Head, ATM Services</t>
+        </is>
+      </c>
+      <c r="C558" t="inlineStr">
+        <is>
+          <t>ZEMEN BANK S.C</t>
+        </is>
+      </c>
+      <c r="D558" t="inlineStr">
+        <is>
+          <t>Banking and Insurance</t>
+        </is>
+      </c>
+      <c r="E558" t="inlineStr">
+        <is>
+          <t>Addis Ababa</t>
+        </is>
+      </c>
+      <c r="F558" t="inlineStr">
+        <is>
+          <t>Office</t>
+        </is>
+      </c>
+      <c r="O558" t="inlineStr">
+        <is>
+          <t>October 5th, 2026</t>
+        </is>
+      </c>
+      <c r="Q558" t="inlineStr">
+        <is>
+          <t>https://ethiojobs.net/job/UYwV987S7G-section-head-atm-services</t>
+        </is>
+      </c>
+      <c r="R558" t="inlineStr">
+        <is>
+          <t>EthioJobs</t>
+        </is>
+      </c>
+      <c r="S558" t="inlineStr">
+        <is>
+          <t>2 hours ago by</t>
+        </is>
+      </c>
+      <c r="T558" t="inlineStr">
+        <is>
+          <t>2026-09-28 15:33:18 UTC</t>
+        </is>
+      </c>
+      <c r="U558" t="inlineStr">
+        <is>
+          <t>listing_only</t>
+        </is>
+      </c>
+    </row>
+    <row r="559">
+      <c r="A559" t="inlineStr">
+        <is>
+          <t>6XUHJDQax4</t>
+        </is>
+      </c>
+      <c r="B559" t="inlineStr">
+        <is>
+          <t>Junior Finance Expert II</t>
+        </is>
+      </c>
+      <c r="C559" t="inlineStr">
+        <is>
+          <t>NATIONAL ELECTION BOARD OF ETHIOPIA(NEBE)</t>
+        </is>
+      </c>
+      <c r="D559" t="inlineStr">
+        <is>
+          <t>Accounting and Finance</t>
+        </is>
+      </c>
+      <c r="E559" t="inlineStr">
+        <is>
+          <t>Addis Ababa</t>
+        </is>
+      </c>
+      <c r="F559" t="inlineStr">
+        <is>
+          <t>Office</t>
+        </is>
+      </c>
+      <c r="G559" t="inlineStr">
+        <is>
+          <t>Mid Level(3-5 years)</t>
+        </is>
+      </c>
+      <c r="H559" t="inlineStr">
+        <is>
+          <t>Full time</t>
+        </is>
+      </c>
+      <c r="I559" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J559" t="inlineStr">
+        <is>
+          <t>and</t>
+        </is>
+      </c>
+      <c r="K559" t="inlineStr">
+        <is>
+          <t>2 years</t>
+        </is>
+      </c>
+      <c r="L559" t="inlineStr">
+        <is>
+          <t>Accounting; Accounting Principles (GAAP), IFRS and ERP; xperience and knowledge of IFMIS, IFRIS is required</t>
+        </is>
+      </c>
+      <c r="O559" t="inlineStr">
+        <is>
+          <t>October 8th, 2026</t>
+        </is>
+      </c>
+      <c r="P559" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      INTERESTED APPLICANTS ARE INVITED TO SEND NON-RETURNABLE:
+Application letter that explains why you fit for the post and updated CV, and Three work related referees;
+Application letter &amp; resume should be saved by full name of Applicants.
+Only short-listed candidates will be contacted for further screening.
+Those who are interested can only apply through the attached link
+https://nebe-election.org/apply  Within 10 days from this announcement.
+Female candidates are encouraged to apply!</t>
+        </is>
+      </c>
+      <c r="Q559" t="inlineStr">
+        <is>
+          <t>https://ethiojobs.net/job/6XUHJDQax4-junior-finance-expert-ii</t>
+        </is>
+      </c>
+      <c r="R559" t="inlineStr">
+        <is>
+          <t>EthioJobs</t>
+        </is>
+      </c>
+      <c r="S559" t="inlineStr">
+        <is>
+          <t>2 hours ago by</t>
+        </is>
+      </c>
+      <c r="T559" t="inlineStr">
+        <is>
+          <t>2026-09-28 15:33:22 UTC</t>
+        </is>
+      </c>
+      <c r="U559" t="inlineStr">
+        <is>
+          <t>dom_render</t>
+        </is>
+      </c>
+    </row>
+    <row r="560">
+      <c r="A560" t="inlineStr">
+        <is>
+          <t>iLsLUngnyh</t>
+        </is>
+      </c>
+      <c r="B560" t="inlineStr">
+        <is>
+          <t>Ticketing Officer</t>
+        </is>
+      </c>
+      <c r="C560" t="inlineStr">
+        <is>
+          <t>NOLAWI TOUR &amp; TRAVEL</t>
+        </is>
+      </c>
+      <c r="D560" t="inlineStr">
+        <is>
+          <t>Social Sciences and Com...; Travel and Tourism</t>
+        </is>
+      </c>
+      <c r="E560" t="inlineStr">
+        <is>
+          <t>Addis Ababa</t>
+        </is>
+      </c>
+      <c r="F560" t="inlineStr">
+        <is>
+          <t>Office</t>
+        </is>
+      </c>
+      <c r="G560" t="inlineStr">
+        <is>
+          <t>Mid Level(3-5 years)</t>
+        </is>
+      </c>
+      <c r="H560" t="inlineStr">
+        <is>
+          <t>Freelance</t>
+        </is>
+      </c>
+      <c r="I560" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="L560" t="inlineStr">
+        <is>
+          <t>Decision-making skills; Communication; Attention to detail; Analytical thinking and problem-solving skills.</t>
+        </is>
+      </c>
+      <c r="O560" t="inlineStr">
+        <is>
+          <t>October 20th, 2026</t>
+        </is>
+      </c>
+      <c r="P560" t="inlineStr">
+        <is>
+          <t>Interested candidates may apply either in person or by email . • In Person: Submit your CV and required documents, along with a non-returnable photocopy, at the office located behind Haya Hulet Debre Damo Hotel, below Arsho Laboratory . • By Email: Send your CV and required documents to theod.visionary@gmail.com For more Information +251977933333/+251968454647</t>
+        </is>
+      </c>
+      <c r="Q560" t="inlineStr">
+        <is>
+          <t>https://ethiojobs.net/job/iLsLUngnyh-ticketing-officer</t>
+        </is>
+      </c>
+      <c r="R560" t="inlineStr">
+        <is>
+          <t>EthioJobs</t>
+        </is>
+      </c>
+      <c r="S560" t="inlineStr">
+        <is>
+          <t>2 hours ago by</t>
+        </is>
+      </c>
+      <c r="T560" t="inlineStr">
+        <is>
+          <t>2026-09-28 15:33:25 UTC</t>
+        </is>
+      </c>
+      <c r="U560" t="inlineStr">
+        <is>
+          <t>dom_render</t>
+        </is>
+      </c>
+    </row>
+    <row r="561">
+      <c r="A561" t="inlineStr">
+        <is>
+          <t>tl8JsjEQCH</t>
+        </is>
+      </c>
+      <c r="B561" t="inlineStr">
+        <is>
+          <t>Senior, District Digital Officer</t>
+        </is>
+      </c>
+      <c r="C561" t="inlineStr">
+        <is>
+          <t>HIJRA BANK S.C</t>
+        </is>
+      </c>
+      <c r="D561" t="inlineStr">
+        <is>
+          <t>Banking and Insurance; Accounting and Finance; Business and Administra...</t>
+        </is>
+      </c>
+      <c r="E561" t="inlineStr">
+        <is>
+          <t>Oromia</t>
+        </is>
+      </c>
+      <c r="F561" t="inlineStr">
+        <is>
+          <t>Office</t>
+        </is>
+      </c>
+      <c r="G561" t="inlineStr">
+        <is>
+          <t>Mid Level(3-5 years)</t>
+        </is>
+      </c>
+      <c r="H561" t="inlineStr">
+        <is>
+          <t>Full time</t>
+        </is>
+      </c>
+      <c r="I561" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="L561" t="inlineStr">
+        <is>
+          <t>Technological &amp; digital literacy; Digital Finance Transformation</t>
+        </is>
+      </c>
+      <c r="O561" t="inlineStr">
+        <is>
+          <t>October 7th, 2026</t>
+        </is>
+      </c>
+      <c r="P561" t="inlineStr">
+        <is>
+          <t>Interested and qualified applicants should apply within ten (10) consecutive calendar days from the date of this announcement through: https://forms.gle/PbNZrXVogg2ky7sd6
+Perks + Benefits
+Fuel
+Housing
+Loan
+Medical Allowance
+Training Opportunities</t>
+        </is>
+      </c>
+      <c r="Q561" t="inlineStr">
+        <is>
+          <t>https://ethiojobs.net/job/tl8JsjEQCH-senior-district-digital-officer</t>
+        </is>
+      </c>
+      <c r="R561" t="inlineStr">
+        <is>
+          <t>EthioJobs</t>
+        </is>
+      </c>
+      <c r="S561" t="inlineStr">
+        <is>
+          <t>2 hours ago by</t>
+        </is>
+      </c>
+      <c r="T561" t="inlineStr">
+        <is>
+          <t>2026-09-28 15:33:28 UTC</t>
+        </is>
+      </c>
+      <c r="U561" t="inlineStr">
+        <is>
+          <t>dom_render</t>
+        </is>
+      </c>
+    </row>
+    <row r="562">
+      <c r="A562" t="inlineStr">
+        <is>
+          <t>5z4gvaz1aB</t>
+        </is>
+      </c>
+      <c r="B562" t="inlineStr">
+        <is>
+          <t>Graduate Internship Program (GIP)</t>
+        </is>
+      </c>
+      <c r="C562" t="inlineStr">
+        <is>
+          <t>EAST AFRICA BOTTLING SHARE COMPANY - COCA COLA</t>
+        </is>
+      </c>
+      <c r="D562" t="inlineStr">
+        <is>
+          <t>Graduate and Management...; Human Resource and Recr...; Sales and Marketing; Engineering</t>
+        </is>
+      </c>
+      <c r="E562" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="F562" t="inlineStr">
+        <is>
+          <t>Office</t>
+        </is>
+      </c>
+      <c r="G562" t="inlineStr">
+        <is>
+          <t>Entry Level (Fresh Graduate)</t>
+        </is>
+      </c>
+      <c r="H562" t="inlineStr">
+        <is>
+          <t>Internship</t>
+        </is>
+      </c>
+      <c r="I562" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J562" t="inlineStr">
+        <is>
+          <t>Bachelor's degree</t>
+        </is>
+      </c>
+      <c r="L562" t="inlineStr">
+        <is>
+          <t>Analytical skills</t>
+        </is>
+      </c>
+      <c r="O562" t="inlineStr">
+        <is>
+          <t>October 7th, 2026</t>
+        </is>
+      </c>
+      <c r="P562" t="inlineStr">
+        <is>
+          <t>Interested and qualified candidates who meet the above requirements are invited to submit their applications through the following link: Application link
+Please note:
+Due to the high volume of applications, we may not be able to respond to all applicants individually.
+Applicants are required to follow our official Telegram channel for updates on their application status, shortlisting results, assessment schedules, and other important recruitment announcements using the link below.
+It is the responsibility of each applicant to regularly check the Telegram channel throughout the recruitment process.
+Official Telegram Channel: CCBAETHIOPIA</t>
+        </is>
+      </c>
+      <c r="Q562" t="inlineStr">
+        <is>
+          <t>https://ethiojobs.net/job/5z4gvaz1aB-graduate-internship-program-gip</t>
+        </is>
+      </c>
+      <c r="R562" t="inlineStr">
+        <is>
+          <t>EthioJobs</t>
+        </is>
+      </c>
+      <c r="S562" t="inlineStr">
+        <is>
+          <t>2 hours ago by</t>
+        </is>
+      </c>
+      <c r="T562" t="inlineStr">
+        <is>
+          <t>2026-09-28 15:33:31 UTC</t>
+        </is>
+      </c>
+      <c r="U562" t="inlineStr">
+        <is>
+          <t>dom_render</t>
+        </is>
+      </c>
+    </row>
+    <row r="563">
+      <c r="A563" t="inlineStr">
+        <is>
+          <t>coyWJwZ3KK</t>
+        </is>
+      </c>
+      <c r="B563" t="inlineStr">
+        <is>
+          <t>Branch Manager I</t>
+        </is>
+      </c>
+      <c r="C563" t="inlineStr">
+        <is>
+          <t>HIJRA BANK S.C</t>
+        </is>
+      </c>
+      <c r="D563" t="inlineStr">
+        <is>
+          <t>Banking and Insurance; Accounting and Finance; Business and Administra...</t>
+        </is>
+      </c>
+      <c r="E563" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="F563" t="inlineStr">
+        <is>
+          <t>Office</t>
+        </is>
+      </c>
+      <c r="G563" t="inlineStr">
+        <is>
+          <t>Senior(5-8 years)</t>
+        </is>
+      </c>
+      <c r="H563" t="inlineStr">
+        <is>
+          <t>Full time</t>
+        </is>
+      </c>
+      <c r="I563" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="L563" t="inlineStr">
+        <is>
+          <t>Market research; Excellent customer service; Leadership &amp; Team Management; Financial control &amp; reporting Treasury &amp; cash management</t>
+        </is>
+      </c>
+      <c r="O563" t="inlineStr">
+        <is>
+          <t>October 7th, 2026</t>
+        </is>
+      </c>
+      <c r="P563" t="inlineStr">
+        <is>
+          <t>Interested and qualified applicants should apply within ten (10) consecutive calendar days from the date of this announcement through: https://forms.gle/PbNZrXVogg2ky7sd6
+Perks + Benefits
+Fuel
+Housing
+Loan
+Medical Allowance
+Training Opportunities</t>
+        </is>
+      </c>
+      <c r="Q563" t="inlineStr">
+        <is>
+          <t>https://ethiojobs.net/job/coyWJwZ3KK-branch-manager-i</t>
+        </is>
+      </c>
+      <c r="R563" t="inlineStr">
+        <is>
+          <t>EthioJobs</t>
+        </is>
+      </c>
+      <c r="S563" t="inlineStr">
+        <is>
+          <t>3 hours ago by</t>
+        </is>
+      </c>
+      <c r="T563" t="inlineStr">
+        <is>
+          <t>2026-09-28 15:33:34 UTC</t>
+        </is>
+      </c>
+      <c r="U563" t="inlineStr">
+        <is>
+          <t>dom_render</t>
+        </is>
+      </c>
+    </row>
+    <row r="564">
+      <c r="A564" t="inlineStr">
+        <is>
+          <t>3FFXWb2EYA</t>
+        </is>
+      </c>
+      <c r="B564" t="inlineStr">
+        <is>
+          <t>Personal &amp; General Service Officer I</t>
+        </is>
+      </c>
+      <c r="C564" t="inlineStr">
+        <is>
+          <t>WAGWAGO BUSINESS GROUP</t>
+        </is>
+      </c>
+      <c r="D564" t="inlineStr">
+        <is>
+          <t>Human Resource and Recr...</t>
+        </is>
+      </c>
+      <c r="E564" t="inlineStr">
+        <is>
+          <t>Addis Ababa</t>
+        </is>
+      </c>
+      <c r="F564" t="inlineStr">
+        <is>
+          <t>Office</t>
+        </is>
+      </c>
+      <c r="G564" t="inlineStr">
+        <is>
+          <t>Junior Level(1-3 years)</t>
+        </is>
+      </c>
+      <c r="H564" t="inlineStr">
+        <is>
+          <t>Full time</t>
+        </is>
+      </c>
+      <c r="I564" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J564" t="inlineStr">
+        <is>
+          <t>Bachelor's degree</t>
+        </is>
+      </c>
+      <c r="K564" t="inlineStr">
+        <is>
+          <t>1-3 years</t>
+        </is>
+      </c>
+      <c r="L564" t="inlineStr">
+        <is>
+          <t>Teamwork; Problem solving; Communication &amp; Negotiation; • Strong coordination and networking skills; Ability to work under pressure and meet deadlines; Ability to multitask and prioritize work</t>
+        </is>
+      </c>
+      <c r="O564" t="inlineStr">
+        <is>
+          <t>October 29th, 2026</t>
+        </is>
+      </c>
+      <c r="P564" t="inlineStr">
+        <is>
+          <t>Candidates who fulfill the above requirements can submit their application through the Company ATS link:
+https://erp.wagwagoelectric.com/jobs/personal-general-service-officer-1096</t>
+        </is>
+      </c>
+      <c r="Q564" t="inlineStr">
+        <is>
+          <t>https://ethiojobs.net/job/3FFXWb2EYA-personal-general-service-officer-i</t>
+        </is>
+      </c>
+      <c r="R564" t="inlineStr">
+        <is>
+          <t>EthioJobs</t>
+        </is>
+      </c>
+      <c r="S564" t="inlineStr">
+        <is>
+          <t>3 hours ago by</t>
+        </is>
+      </c>
+      <c r="T564" t="inlineStr">
+        <is>
+          <t>2026-09-28 15:33:40 UTC</t>
+        </is>
+      </c>
+      <c r="U564" t="inlineStr">
+        <is>
+          <t>dom_render</t>
+        </is>
+      </c>
+    </row>
+    <row r="565">
+      <c r="A565" t="inlineStr">
+        <is>
+          <t>xpZ3NtZwqA</t>
+        </is>
+      </c>
+      <c r="B565" t="inlineStr">
+        <is>
+          <t>Branch Operation Supervisor</t>
+        </is>
+      </c>
+      <c r="C565" t="inlineStr">
+        <is>
+          <t>HIJRA BANK S.C</t>
+        </is>
+      </c>
+      <c r="D565" t="inlineStr">
+        <is>
+          <t>Banking and Insurance; Accounting and Finance; Business and Administra...</t>
+        </is>
+      </c>
+      <c r="E565" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="F565" t="inlineStr">
+        <is>
+          <t>Office</t>
+        </is>
+      </c>
+      <c r="G565" t="inlineStr">
+        <is>
+          <t>Senior(5-8 years)</t>
+        </is>
+      </c>
+      <c r="H565" t="inlineStr">
+        <is>
+          <t>Full time</t>
+        </is>
+      </c>
+      <c r="I565" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="L565" t="inlineStr">
+        <is>
+          <t>Account management; Excellent customer service; Audit &amp; Compliance Management; Financial control &amp; reporting Treasury &amp; cash management</t>
+        </is>
+      </c>
+      <c r="O565" t="inlineStr">
+        <is>
+          <t>October 7th, 2026</t>
+        </is>
+      </c>
+      <c r="P565" t="inlineStr">
+        <is>
+          <t>Interested and qualified applicants should apply within ten (10) consecutive calendar days from the date of this announcement through: https://forms.gle/PbNZrXVogg2ky7sd6
+Perks + Benefits
+Fuel
+Housing
+Loan
+Medical Allowance
+Training Opportunities</t>
+        </is>
+      </c>
+      <c r="Q565" t="inlineStr">
+        <is>
+          <t>https://ethiojobs.net/job/xpZ3NtZwqA-branch-operation-supervisor</t>
+        </is>
+      </c>
+      <c r="R565" t="inlineStr">
+        <is>
+          <t>EthioJobs</t>
+        </is>
+      </c>
+      <c r="S565" t="inlineStr">
+        <is>
+          <t>3 hours ago by</t>
+        </is>
+      </c>
+      <c r="T565" t="inlineStr">
+        <is>
+          <t>2026-09-28 15:33:43 UTC</t>
+        </is>
+      </c>
+      <c r="U565" t="inlineStr">
+        <is>
+          <t>dom_render</t>
+        </is>
+      </c>
+    </row>
+    <row r="566">
+      <c r="A566" t="inlineStr">
+        <is>
+          <t>COCIxGX0qY</t>
+        </is>
+      </c>
+      <c r="B566" t="inlineStr">
+        <is>
+          <t>Senior Customer Service Officer</t>
+        </is>
+      </c>
+      <c r="C566" t="inlineStr">
+        <is>
+          <t>HIJRA BANK S.C</t>
+        </is>
+      </c>
+      <c r="D566" t="inlineStr">
+        <is>
+          <t>Banking and Insurance; Accounting and Finance; Business and Administra...</t>
+        </is>
+      </c>
+      <c r="E566" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="F566" t="inlineStr">
+        <is>
+          <t>Office</t>
+        </is>
+      </c>
+      <c r="G566" t="inlineStr">
+        <is>
+          <t>Mid Level(3-5 years)</t>
+        </is>
+      </c>
+      <c r="H566" t="inlineStr">
+        <is>
+          <t>Full time</t>
+        </is>
+      </c>
+      <c r="I566" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="L566" t="inlineStr">
+        <is>
+          <t>Marketing management, Business Management; Excellent customer service; Financial control &amp; reporting Treasury &amp; cash management</t>
+        </is>
+      </c>
+      <c r="O566" t="inlineStr">
+        <is>
+          <t>October 7th, 2026</t>
+        </is>
+      </c>
+      <c r="P566" t="inlineStr">
+        <is>
+          <t>Interested and qualified applicants should apply within ten (10) consecutive calendar days from the date of this announcement through: https://forms.gle/PbNZrXVogg2ky7sd6
+Perks + Benefits
+Fuel
+Housing
+Loan
+Medical Allowance
+Training Opportunities</t>
+        </is>
+      </c>
+      <c r="Q566" t="inlineStr">
+        <is>
+          <t>https://ethiojobs.net/job/COCIxGX0qY-senior-customer-service-officer</t>
+        </is>
+      </c>
+      <c r="R566" t="inlineStr">
+        <is>
+          <t>EthioJobs</t>
+        </is>
+      </c>
+      <c r="S566" t="inlineStr">
+        <is>
+          <t>3 hours ago by</t>
+        </is>
+      </c>
+      <c r="T566" t="inlineStr">
+        <is>
+          <t>2026-09-28 15:33:46 UTC</t>
+        </is>
+      </c>
+      <c r="U566" t="inlineStr">
+        <is>
+          <t>dom_render</t>
+        </is>
+      </c>
+    </row>
+    <row r="567">
+      <c r="A567" t="inlineStr">
+        <is>
+          <t>9nsNnDhxRZ</t>
+        </is>
+      </c>
+      <c r="B567" t="inlineStr">
+        <is>
+          <t>Techinichal and Oprational Manager (Pharmacy sector)</t>
+        </is>
+      </c>
+      <c r="C567" t="inlineStr">
+        <is>
+          <t>ANNAM MARKETING SOLUTION PLC</t>
+        </is>
+      </c>
+      <c r="D567" t="inlineStr">
+        <is>
+          <t>Pharmaceutical; Natural Sciences</t>
+        </is>
+      </c>
+      <c r="E567" t="inlineStr">
+        <is>
+          <t>Addis Ababa</t>
+        </is>
+      </c>
+      <c r="F567" t="inlineStr">
+        <is>
+          <t>Office</t>
+        </is>
+      </c>
+      <c r="G567" t="inlineStr">
+        <is>
+          <t>Mid Level(3-5 years)</t>
+        </is>
+      </c>
+      <c r="H567" t="inlineStr">
+        <is>
+          <t>Full time</t>
+        </is>
+      </c>
+      <c r="I567" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K567" t="inlineStr">
+        <is>
+          <t>3 years</t>
+        </is>
+      </c>
+      <c r="L567" t="inlineStr">
+        <is>
+          <t>Communication</t>
+        </is>
+      </c>
+      <c r="O567" t="inlineStr">
+        <is>
+          <t>October 29th, 2026</t>
+        </is>
+      </c>
+      <c r="P567" t="inlineStr">
+        <is>
+          <t>Interested applicant shall submit CV, copy of academic documents, copy of testimonials, application letters in person at Bole Friendship Building, Office No. 804/3. Phone No.: 0911551022
+Application date: 10 Days as of the vacancy announcement.</t>
+        </is>
+      </c>
+      <c r="Q567" t="inlineStr">
+        <is>
+          <t>https://ethiojobs.net/job/9nsNnDhxRZ-techinichal-and-oprational-manager-pharmacy-sector</t>
+        </is>
+      </c>
+      <c r="R567" t="inlineStr">
+        <is>
+          <t>EthioJobs</t>
+        </is>
+      </c>
+      <c r="S567" t="inlineStr">
+        <is>
+          <t>3 hours ago by</t>
+        </is>
+      </c>
+      <c r="T567" t="inlineStr">
+        <is>
+          <t>2026-09-28 15:33:49 UTC</t>
+        </is>
+      </c>
+      <c r="U567" t="inlineStr">
+        <is>
+          <t>dom_render</t>
+        </is>
+      </c>
+    </row>
+    <row r="568">
+      <c r="A568" t="inlineStr">
+        <is>
+          <t>WpYm5vEGeL</t>
+        </is>
+      </c>
+      <c r="B568" t="inlineStr">
+        <is>
+          <t>FINANCE AND HR ADMINISTRATION OFFICER</t>
+        </is>
+      </c>
+      <c r="C568" t="inlineStr">
+        <is>
+          <t>ZEWDITU GETACHEW FOUNDATION</t>
+        </is>
+      </c>
+      <c r="D568" t="inlineStr">
+        <is>
+          <t>Accounting and Finance; Business and Administra...</t>
+        </is>
+      </c>
+      <c r="E568" t="inlineStr">
+        <is>
+          <t>Addis Ababa</t>
+        </is>
+      </c>
+      <c r="F568" t="inlineStr">
+        <is>
+          <t>Office</t>
+        </is>
+      </c>
+      <c r="G568" t="inlineStr">
+        <is>
+          <t>Junior Level(1-3 years)</t>
+        </is>
+      </c>
+      <c r="H568" t="inlineStr">
+        <is>
+          <t>Full time</t>
+        </is>
+      </c>
+      <c r="I568" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K568" t="inlineStr">
+        <is>
+          <t>1-3 years</t>
+        </is>
+      </c>
+      <c r="L568" t="inlineStr">
+        <is>
+          <t>Communication; Attention to detail; Problem solving</t>
+        </is>
+      </c>
+      <c r="O568" t="inlineStr">
+        <is>
+          <t>October 29th, 2026</t>
+        </is>
+      </c>
+      <c r="P568" t="inlineStr">
+        <is>
+          <t>Contact Address: Zewditu Getachew Foundation, Kirkos Sub-City, Woreda 01, Bambis, Afework Building, Office -205, tsigegm@zewditugetachew.org, Tel: +252911242095</t>
+        </is>
+      </c>
+      <c r="Q568" t="inlineStr">
+        <is>
+          <t>https://ethiojobs.net/job/WpYm5vEGeL-finance-and-hr-administration-officer</t>
+        </is>
+      </c>
+      <c r="R568" t="inlineStr">
+        <is>
+          <t>EthioJobs</t>
+        </is>
+      </c>
+      <c r="S568" t="inlineStr">
+        <is>
+          <t>3 hours ago by</t>
+        </is>
+      </c>
+      <c r="T568" t="inlineStr">
+        <is>
+          <t>2026-09-28 15:33:52 UTC</t>
+        </is>
+      </c>
+      <c r="U568" t="inlineStr">
+        <is>
+          <t>dom_render</t>
+        </is>
+      </c>
+    </row>
+    <row r="569">
+      <c r="A569" t="inlineStr">
+        <is>
+          <t>xcSAOWy1mE</t>
+        </is>
+      </c>
+      <c r="B569" t="inlineStr">
+        <is>
+          <t>Customer Service Officer II</t>
+        </is>
+      </c>
+      <c r="C569" t="inlineStr">
+        <is>
+          <t>HIJRA BANK S.C</t>
+        </is>
+      </c>
+      <c r="D569" t="inlineStr">
+        <is>
+          <t>Banking and Insurance; Accounting and Finance; Business and Administra...</t>
+        </is>
+      </c>
+      <c r="E569" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="F569" t="inlineStr">
+        <is>
+          <t>Office</t>
+        </is>
+      </c>
+      <c r="G569" t="inlineStr">
+        <is>
+          <t>Junior Level(1-3 years)</t>
+        </is>
+      </c>
+      <c r="H569" t="inlineStr">
+        <is>
+          <t>Full time</t>
+        </is>
+      </c>
+      <c r="I569" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="K569" t="inlineStr">
+        <is>
+          <t>1-3 years</t>
+        </is>
+      </c>
+      <c r="L569" t="inlineStr">
+        <is>
+          <t>Attention to detail; Excellent customer service</t>
+        </is>
+      </c>
+      <c r="O569" t="inlineStr">
+        <is>
+          <t>October 7th, 2026</t>
+        </is>
+      </c>
+      <c r="P569" t="inlineStr">
+        <is>
+          <t>Interested and qualified applicants should apply within ten (10) consecutive calendar days from the date of this announcement through:
+Perks + Benefits
+Fuel
+Housing
+Loan
+Medical Allowance
+Training Opportunities</t>
+        </is>
+      </c>
+      <c r="Q569" t="inlineStr">
+        <is>
+          <t>https://ethiojobs.net/job/xcSAOWy1mE-customer-service-officer-ii</t>
+        </is>
+      </c>
+      <c r="R569" t="inlineStr">
+        <is>
+          <t>EthioJobs</t>
+        </is>
+      </c>
+      <c r="S569" t="inlineStr">
+        <is>
+          <t>3 hours ago by</t>
+        </is>
+      </c>
+      <c r="T569" t="inlineStr">
+        <is>
+          <t>2026-09-28 15:33:55 UTC</t>
+        </is>
+      </c>
+      <c r="U569" t="inlineStr">
+        <is>
+          <t>dom_render</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:U1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -51760,7 +54383,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -51856,6 +54479,19 @@
       </c>
       <c r="C7" t="n">
         <v>540</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-09-28 15:33:57 UTC</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>28</v>
+      </c>
+      <c r="C8" t="n">
+        <v>568</v>
       </c>
     </row>
   </sheetData>

</xml_diff>